<commit_message>
Daily EOD data and reports for 2026-09-02
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260902.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260902.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.865</v>
+        <v>1.895</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.075</v>
+        <v>-0.045</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-3.87%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>285682.57</v>
+        <v>290277.99</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-11488.57</v>
+        <v>-6893.14</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.415</v>
+        <v>2.47</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.045</v>
+        <v>0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.83%</t>
+          <t>0.41%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>169050</v>
+        <v>172900</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-3150</v>
+        <v>700</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>64.64</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-2.2</v>
+        <v>-2.19</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.28%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>9000</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>581760</v>
+        <v>581850</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-19800</v>
+        <v>-19710</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.004</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>176.36</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-176.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>158.68</v>
+        <v>159.32</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.47</v>
+        <v>0.17</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.30%</t>
+          <t>0.11%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.045</v>
+        <v>-0.02</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-4.59%</t>
+          <t>-2.04%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9350</v>
+        <v>9600</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-450</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>171.885</v>
+        <v>173.85</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.425</v>
+        <v>1.54</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.25%</t>
+          <t>0.89%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>687540</v>
+        <v>695400</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-1700</v>
+        <v>6160</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.27</v>
+        <v>0.265</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.85%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5400</v>
+        <v>5300</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.005</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-4.35%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1035.32</v>
+        <v>1129.44</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-47.06</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.098</v>
+        <v>0.099</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.002</v>
+        <v>-0.001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-2.00%</t>
+          <t>-1.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-12</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.36</v>
+        <v>34.39</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>0.09%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.19</v>
+        <v>33.08</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.49</v>
+        <v>0.38</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>1.16%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42748.72</v>
+        <v>42607.04</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>631.12</v>
+        <v>489.44</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1783154.6</v>
+        <v>1799834.83</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-104818.74</v>
+        <v>-88138.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>